<commit_message>
Suma también Costo anual (USD) al consolidar registros de un usuario
Corrige la consolidación: los montos que se suman por usuario incluyen
Costo anual (USD) además de Facturado USD, Facturado MXN y Presupuesto
Ops. Ej.: oguzmant (240 + 960) = 1200. Los cuatro montos reconcilian con
el total original (Costo anual 27,120). Los campos descriptivos y la
Fecha siguen tomándose del último registro.

Verificado con navegador headless: dashboard y Excel exportado coinciden
con el script Python.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGhbBicCw2EmxaVu1AmQRf
</commit_message>
<xml_diff>
--- a/Analisis_Usabilidad_Final.xlsx
+++ b/Analisis_Usabilidad_Final.xlsx
@@ -4113,7 +4113,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="4">
-        <v>960</v>
+        <v>1200</v>
       </c>
       <c r="E9" s="4">
         <v>1125.93</v>
@@ -4233,7 +4233,7 @@
         <v>85</v>
       </c>
       <c r="D15" s="6">
-        <v>26880</v>
+        <v>27120</v>
       </c>
       <c r="E15" s="6">
         <v>24351.75</v>
@@ -5637,7 +5637,7 @@
         <v>1</v>
       </c>
       <c r="I16">
-        <v>960</v>
+        <v>1200</v>
       </c>
       <c r="J16">
         <v>1125.93</v>

</xml_diff>

<commit_message>
Costo por Nivel refleja el costo total del proyecto (\$27,120 USD)
El costo por nivel de uso se calcula ahora sobre el master COMPLETO (todos
los usuarios consolidados, incluidas las licencias de equipo sin usuario
nombrado como dx_chatgpt). Así el total es consistente con el costo real:
Costo anual \$27,120 USD y Facturado \$462,683.25 MXN.

Las vistas de usabilidad (Usabilidad Usuarios, Resumen Niveles, % Uso por
Team, Consumo Presup. Ops, Análisis Detallado) siguen usando el master
vigente (Cantidad lic > 0). La licencia de equipo sin uso cae en Nulo y
suma al monto ocioso, que es la lectura correcta.

Verificado con navegador headless: dashboard y Excel exportado coinciden
con el script Python (Productivo \$232,617.07 / Ocioso \$154,377.40 /
En adopción \$75,688.78 MXN; Costo anual total \$27,120).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGhbBicCw2EmxaVu1AmQRf
</commit_message>
<xml_diff>
--- a/Analisis_Usabilidad_Final.xlsx
+++ b/Analisis_Usabilidad_Final.xlsx
@@ -690,7 +690,7 @@
     <t>Costo por nivel de uso — monto ocioso vs productivo</t>
   </si>
   <si>
-    <t>Productivo (Muy Alto/Alto/Medio): 232,617.07 MXN   |   Ocioso (Bajo/Nulo): 131,577.40 MXN   |   En adopción (Reciente): 75,688.78 MXN</t>
+    <t>Productivo (Muy Alto/Alto/Medio): 232,617.07 MXN   |   Ocioso (Bajo/Nulo): 154,377.40 MXN   |   En adopción (Reciente): 75,688.78 MXN</t>
   </si>
   <si>
     <t>Resumen de aprovechamiento</t>
@@ -1800,7 +1800,7 @@
                   <c:v>88455.735</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>43121.6685</c:v>
+                  <c:v>65921.6685</c:v>
                 </c:pt>
                 <c:pt idx="5">
                   <c:v>75688.78</c:v>
@@ -1943,7 +1943,7 @@
                   <c:v>75688.78</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>131577.4035</c:v>
+                  <c:v>154377.4035</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -6365,7 +6365,7 @@
         <v>69082.98666666666</v>
       </c>
       <c r="F6">
-        <v>15.7</v>
+        <v>14.9</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -6385,7 +6385,7 @@
         <v>96989.97291666667</v>
       </c>
       <c r="F7">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -6405,7 +6405,7 @@
         <v>66544.10691666667</v>
       </c>
       <c r="F8">
-        <v>15.1</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -6425,7 +6425,7 @@
         <v>88455.735</v>
       </c>
       <c r="F9">
-        <v>20.1</v>
+        <v>19.1</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -6436,16 +6436,16 @@
         <v>218</v>
       </c>
       <c r="C10">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D10" s="4">
-        <v>2400</v>
+        <v>3600</v>
       </c>
       <c r="E10" s="4">
-        <v>43121.6685</v>
+        <v>65921.6685</v>
       </c>
       <c r="F10">
-        <v>9.800000000000001</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -6465,7 +6465,7 @@
         <v>75688.78</v>
       </c>
       <c r="F11">
-        <v>17.2</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -6474,13 +6474,13 @@
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D12" s="6">
-        <v>25920</v>
+        <v>27120</v>
       </c>
       <c r="E12" s="6">
-        <v>439883.25</v>
+        <v>462683.25</v>
       </c>
       <c r="F12" s="6">
         <v>100</v>
@@ -6522,7 +6522,7 @@
         <v>13200</v>
       </c>
       <c r="E15" s="4">
-        <v>52.9</v>
+        <v>50.3</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -6539,7 +6539,7 @@
         <v>5280</v>
       </c>
       <c r="E16" s="4">
-        <v>17.2</v>
+        <v>16.4</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -6547,16 +6547,16 @@
         <v>218</v>
       </c>
       <c r="B17">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C17">
-        <v>131577.4035</v>
+        <v>154377.4035</v>
       </c>
       <c r="D17" s="4">
-        <v>7440</v>
+        <v>8640</v>
       </c>
       <c r="E17" s="4">
-        <v>29.9</v>
+        <v>33.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Descarta usabilidad sin última conexión (además de conexión previa a la asignación)
La usabilidad solo se considera válida si existe Last Active y es posterior
o igual a la fecha de asignación. Se descarta el registro de uso (aunque
tenga Days Active u otras métricas) cuando no hay última conexión o cuando
es anterior a la fecha de asignación. En estos datos afecta a 11 registros
(p. ej. jdasilva: Days Active 2 sin Last Active -> se descarta, queda en 0).

Verificado con navegador headless y el script Python (coinciden): 11
usabilidades descartadas, 69 usuarios con uso válido, niveles idénticos.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGhbBicCw2EmxaVu1AmQRf
</commit_message>
<xml_diff>
--- a/Analisis_Usabilidad_Final.xlsx
+++ b/Analisis_Usabilidad_Final.xlsx
@@ -186,150 +186,150 @@
     <t xml:space="preserve">Emma Alguera  </t>
   </si>
   <si>
+    <t>Alfonso Cueto</t>
+  </si>
+  <si>
+    <t>Omar Guzman</t>
+  </si>
+  <si>
+    <t>Bernardo González</t>
+  </si>
+  <si>
+    <t>Procurement Team</t>
+  </si>
+  <si>
+    <t>Sebastián González García</t>
+  </si>
+  <si>
+    <t>Hector Huerta</t>
+  </si>
+  <si>
+    <t>Ramiro Vazquez Vera</t>
+  </si>
+  <si>
+    <t>Jose Ivan Ramirez</t>
+  </si>
+  <si>
+    <t>Lizbeth Aguilar Morales</t>
+  </si>
+  <si>
+    <t>Aniver Chino Marcelino</t>
+  </si>
+  <si>
+    <t>Javier Loeza</t>
+  </si>
+  <si>
+    <t>Daniela Mondragon Corona</t>
+  </si>
+  <si>
+    <t>Victor Iván Soto Guerra</t>
+  </si>
+  <si>
+    <t>Miguel Angel Garrido Castaneda</t>
+  </si>
+  <si>
+    <t>Joaquin Calvo Leon</t>
+  </si>
+  <si>
+    <t>Jonathan Ramón</t>
+  </si>
+  <si>
+    <t>Jesus Morales Enciso</t>
+  </si>
+  <si>
+    <t>Edgar Fidel Salinas Espinoza</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Talia Maciel  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ricardo Laiseca  </t>
+  </si>
+  <si>
+    <t>Marco Espinosa</t>
+  </si>
+  <si>
+    <t>Ricardo Santiago</t>
+  </si>
+  <si>
+    <t>Mercedes Morales</t>
+  </si>
+  <si>
+    <t>Hector Espejel</t>
+  </si>
+  <si>
+    <t>Bruno Juanes</t>
+  </si>
+  <si>
+    <t>Maghandi Suarez</t>
+  </si>
+  <si>
+    <t>Marketing Team</t>
+  </si>
+  <si>
+    <t>Gustavo Gonzalez Martinez</t>
+  </si>
+  <si>
+    <t>Sandy Areli Monroy</t>
+  </si>
+  <si>
+    <t>Juan Carlos Morales Leon</t>
+  </si>
+  <si>
+    <t>Erwin Ordonez Velazquez</t>
+  </si>
+  <si>
+    <t>Nathalie Reyes</t>
+  </si>
+  <si>
+    <t>Raul Jaimes Martin</t>
+  </si>
+  <si>
+    <t>Luis Montes</t>
+  </si>
+  <si>
+    <t>José Ríos Alonso</t>
+  </si>
+  <si>
+    <t>Christian Jesus Ocampo Arce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rodrigo Galindo Mello </t>
+  </si>
+  <si>
+    <t>Aldo Romero</t>
+  </si>
+  <si>
+    <t>Gerardo Tellez</t>
+  </si>
+  <si>
+    <t>Rafael Sánchez</t>
+  </si>
+  <si>
+    <t>Rafael Hernández</t>
+  </si>
+  <si>
+    <t>Abraham Espinal</t>
+  </si>
+  <si>
+    <t>Jonathan Vallejo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Olga Badillo </t>
+  </si>
+  <si>
+    <t>Edwin Medina</t>
+  </si>
+  <si>
+    <t>Javier Reyes</t>
+  </si>
+  <si>
+    <t>Armando Beltran</t>
+  </si>
+  <si>
     <t>José Da Silva</t>
   </si>
   <si>
-    <t>Alfonso Cueto</t>
-  </si>
-  <si>
-    <t>Omar Guzman</t>
-  </si>
-  <si>
-    <t>Bernardo González</t>
-  </si>
-  <si>
-    <t>Procurement Team</t>
-  </si>
-  <si>
-    <t>Sebastián González García</t>
-  </si>
-  <si>
-    <t>Hector Huerta</t>
-  </si>
-  <si>
-    <t>Ramiro Vazquez Vera</t>
-  </si>
-  <si>
-    <t>Jose Ivan Ramirez</t>
-  </si>
-  <si>
-    <t>Lizbeth Aguilar Morales</t>
-  </si>
-  <si>
-    <t>Aniver Chino Marcelino</t>
-  </si>
-  <si>
-    <t>Javier Loeza</t>
-  </si>
-  <si>
-    <t>Daniela Mondragon Corona</t>
-  </si>
-  <si>
-    <t>Victor Iván Soto Guerra</t>
-  </si>
-  <si>
-    <t>Miguel Angel Garrido Castaneda</t>
-  </si>
-  <si>
-    <t>Joaquin Calvo Leon</t>
-  </si>
-  <si>
-    <t>Jonathan Ramón</t>
-  </si>
-  <si>
-    <t>Jesus Morales Enciso</t>
-  </si>
-  <si>
-    <t>Edgar Fidel Salinas Espinoza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Talia Maciel  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ricardo Laiseca  </t>
-  </si>
-  <si>
-    <t>Marco Espinosa</t>
-  </si>
-  <si>
-    <t>Ricardo Santiago</t>
-  </si>
-  <si>
-    <t>Mercedes Morales</t>
-  </si>
-  <si>
-    <t>Hector Espejel</t>
-  </si>
-  <si>
-    <t>Bruno Juanes</t>
-  </si>
-  <si>
-    <t>Maghandi Suarez</t>
-  </si>
-  <si>
-    <t>Marketing Team</t>
-  </si>
-  <si>
-    <t>Gustavo Gonzalez Martinez</t>
-  </si>
-  <si>
-    <t>Sandy Areli Monroy</t>
-  </si>
-  <si>
-    <t>Juan Carlos Morales Leon</t>
-  </si>
-  <si>
-    <t>Erwin Ordonez Velazquez</t>
-  </si>
-  <si>
-    <t>Nathalie Reyes</t>
-  </si>
-  <si>
-    <t>Raul Jaimes Martin</t>
-  </si>
-  <si>
-    <t>Luis Montes</t>
-  </si>
-  <si>
-    <t>José Ríos Alonso</t>
-  </si>
-  <si>
-    <t>Christian Jesus Ocampo Arce</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rodrigo Galindo Mello </t>
-  </si>
-  <si>
-    <t>Aldo Romero</t>
-  </si>
-  <si>
-    <t>Gerardo Tellez</t>
-  </si>
-  <si>
-    <t>Rafael Sánchez</t>
-  </si>
-  <si>
-    <t>Rafael Hernández</t>
-  </si>
-  <si>
-    <t>Abraham Espinal</t>
-  </si>
-  <si>
-    <t>Jonathan Vallejo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Olga Badillo </t>
-  </si>
-  <si>
-    <t>Edwin Medina</t>
-  </si>
-  <si>
-    <t>Javier Reyes</t>
-  </si>
-  <si>
-    <t>Armando Beltran</t>
-  </si>
-  <si>
     <t>Ossiel Cruz Velazquez</t>
   </si>
   <si>
@@ -441,150 +441,150 @@
     <t>ealguera@kio.tech</t>
   </si>
   <si>
+    <t>acueto@kio.tech</t>
+  </si>
+  <si>
+    <t>oguzmant@kio.tech</t>
+  </si>
+  <si>
+    <t>jbgonzalez@kio.tech</t>
+  </si>
+  <si>
+    <t>compras_proyectos@kio.tech</t>
+  </si>
+  <si>
+    <t>sgonzalezg@kio.tech</t>
+  </si>
+  <si>
+    <t>hhuerta@kio.tech</t>
+  </si>
+  <si>
+    <t>rvazquez@kio.tech</t>
+  </si>
+  <si>
+    <t>jramirezl@kio.tech</t>
+  </si>
+  <si>
+    <t>laguilar@kio.tech</t>
+  </si>
+  <si>
+    <t>achino@kio.tech</t>
+  </si>
+  <si>
+    <t>jloeza@kio.tech</t>
+  </si>
+  <si>
+    <t>dmondragon@kio.tech</t>
+  </si>
+  <si>
+    <t>vsoto@kio.tech</t>
+  </si>
+  <si>
+    <t>mgarrido@kio.tech</t>
+  </si>
+  <si>
+    <t>jcalvo@kio.tech</t>
+  </si>
+  <si>
+    <t>jramon@kio.tech</t>
+  </si>
+  <si>
+    <t>jmoralese@kio.tech</t>
+  </si>
+  <si>
+    <t>esalinas@kio.tech</t>
+  </si>
+  <si>
+    <t>tmaciel@kio.tech</t>
+  </si>
+  <si>
+    <t>rilaiseca@kio.tech</t>
+  </si>
+  <si>
+    <t>mespinosa@kio.tech</t>
+  </si>
+  <si>
+    <t>rsantiago@kio.tech</t>
+  </si>
+  <si>
+    <t>mmoralesl@kio.tech</t>
+  </si>
+  <si>
+    <t>hespejel@kio.tech</t>
+  </si>
+  <si>
+    <t>bjuanes@kio.tech</t>
+  </si>
+  <si>
+    <t>msuarezp@kio.tech</t>
+  </si>
+  <si>
+    <t>marketing@kio.tech</t>
+  </si>
+  <si>
+    <t>ggonzalez@kio.tech</t>
+  </si>
+  <si>
+    <t>smonroy@kio.tech</t>
+  </si>
+  <si>
+    <t>jcmorales@kio.tech</t>
+  </si>
+  <si>
+    <t>eordonez@kio.tech</t>
+  </si>
+  <si>
+    <t>nreyesz@kio.tech</t>
+  </si>
+  <si>
+    <t>rjaimes@kio.tech</t>
+  </si>
+  <si>
+    <t>lmontes@kio.tech</t>
+  </si>
+  <si>
+    <t>jriosa@kio.tech</t>
+  </si>
+  <si>
+    <t>cocampo@kio.tech</t>
+  </si>
+  <si>
+    <t>rgalindo@kio.tech</t>
+  </si>
+  <si>
+    <t>aromero@kio.tech</t>
+  </si>
+  <si>
+    <t>gtellez@kio.tech</t>
+  </si>
+  <si>
+    <t>rsanchezo@kio.tech</t>
+  </si>
+  <si>
+    <t>rhernandezb@kio.tech</t>
+  </si>
+  <si>
+    <t>aespinal@kio.tech</t>
+  </si>
+  <si>
+    <t>jjvallejo@kio.tech</t>
+  </si>
+  <si>
+    <t>obadillo@kio.tech</t>
+  </si>
+  <si>
+    <t>emedina@kio.tech</t>
+  </si>
+  <si>
+    <t>jreyes@kio.tech</t>
+  </si>
+  <si>
+    <t>abeltran@kio.tech</t>
+  </si>
+  <si>
     <t>jdasilva@kio.tech</t>
   </si>
   <si>
-    <t>acueto@kio.tech</t>
-  </si>
-  <si>
-    <t>oguzmant@kio.tech</t>
-  </si>
-  <si>
-    <t>jbgonzalez@kio.tech</t>
-  </si>
-  <si>
-    <t>compras_proyectos@kio.tech</t>
-  </si>
-  <si>
-    <t>sgonzalezg@kio.tech</t>
-  </si>
-  <si>
-    <t>hhuerta@kio.tech</t>
-  </si>
-  <si>
-    <t>rvazquez@kio.tech</t>
-  </si>
-  <si>
-    <t>jramirezl@kio.tech</t>
-  </si>
-  <si>
-    <t>laguilar@kio.tech</t>
-  </si>
-  <si>
-    <t>achino@kio.tech</t>
-  </si>
-  <si>
-    <t>jloeza@kio.tech</t>
-  </si>
-  <si>
-    <t>dmondragon@kio.tech</t>
-  </si>
-  <si>
-    <t>vsoto@kio.tech</t>
-  </si>
-  <si>
-    <t>mgarrido@kio.tech</t>
-  </si>
-  <si>
-    <t>jcalvo@kio.tech</t>
-  </si>
-  <si>
-    <t>jramon@kio.tech</t>
-  </si>
-  <si>
-    <t>jmoralese@kio.tech</t>
-  </si>
-  <si>
-    <t>esalinas@kio.tech</t>
-  </si>
-  <si>
-    <t>tmaciel@kio.tech</t>
-  </si>
-  <si>
-    <t>rilaiseca@kio.tech</t>
-  </si>
-  <si>
-    <t>mespinosa@kio.tech</t>
-  </si>
-  <si>
-    <t>rsantiago@kio.tech</t>
-  </si>
-  <si>
-    <t>mmoralesl@kio.tech</t>
-  </si>
-  <si>
-    <t>hespejel@kio.tech</t>
-  </si>
-  <si>
-    <t>bjuanes@kio.tech</t>
-  </si>
-  <si>
-    <t>msuarezp@kio.tech</t>
-  </si>
-  <si>
-    <t>marketing@kio.tech</t>
-  </si>
-  <si>
-    <t>ggonzalez@kio.tech</t>
-  </si>
-  <si>
-    <t>smonroy@kio.tech</t>
-  </si>
-  <si>
-    <t>jcmorales@kio.tech</t>
-  </si>
-  <si>
-    <t>eordonez@kio.tech</t>
-  </si>
-  <si>
-    <t>nreyesz@kio.tech</t>
-  </si>
-  <si>
-    <t>rjaimes@kio.tech</t>
-  </si>
-  <si>
-    <t>lmontes@kio.tech</t>
-  </si>
-  <si>
-    <t>jriosa@kio.tech</t>
-  </si>
-  <si>
-    <t>cocampo@kio.tech</t>
-  </si>
-  <si>
-    <t>rgalindo@kio.tech</t>
-  </si>
-  <si>
-    <t>aromero@kio.tech</t>
-  </si>
-  <si>
-    <t>gtellez@kio.tech</t>
-  </si>
-  <si>
-    <t>rsanchezo@kio.tech</t>
-  </si>
-  <si>
-    <t>rhernandezb@kio.tech</t>
-  </si>
-  <si>
-    <t>aespinal@kio.tech</t>
-  </si>
-  <si>
-    <t>jjvallejo@kio.tech</t>
-  </si>
-  <si>
-    <t>obadillo@kio.tech</t>
-  </si>
-  <si>
-    <t>emedina@kio.tech</t>
-  </si>
-  <si>
-    <t>jreyes@kio.tech</t>
-  </si>
-  <si>
-    <t>abeltran@kio.tech</t>
-  </si>
-  <si>
     <t>ocruzv@kio.tech</t>
   </si>
   <si>
@@ -699,7 +699,7 @@
     <t>Costo por nivel de uso — monto ocioso vs productivo</t>
   </si>
   <si>
-    <t>Productivo (Muy Alto/Alto/Medio): 276,279.81 MXN   |   Ocioso (Bajo/Nulo): 141,129.76 MXN   |   En adopción (Reciente): 45,273.68 MXN</t>
+    <t>Productivo (Muy Alto/Alto/Medio): 272,848.95 MXN   |   Ocioso (Bajo/Nulo): 141,129.76 MXN   |   En adopción (Reciente): 48,704.54 MXN</t>
   </si>
   <si>
     <t>Resumen de aprovechamiento</t>
@@ -1494,7 +1494,7 @@
                   <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>22</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>22</c:v>
@@ -1503,7 +1503,7 @@
                   <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>13</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1621,10 +1621,10 @@
                   <c:v>Marketing</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>Dir Ops</c:v>
+                  <c:v>Dirección</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>Dirección</c:v>
+                  <c:v>Dir Ops</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>Ops - Plataformas</c:v>
@@ -1666,10 +1666,10 @@
                   <c:v>41.2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>40.8</c:v>
+                  <c:v>37.6</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>37.6</c:v>
+                  <c:v>33.6</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>29.6</c:v>
@@ -1851,7 +1851,7 @@
                   <c:v>93794.42941666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>104004.2029166667</c:v>
+                  <c:v>100573.3444166667</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>106863.8185</c:v>
@@ -1860,7 +1860,7 @@
                   <c:v>34265.94425</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>45273.67975</c:v>
+                  <c:v>48704.53825</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1994,10 +1994,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>276279.8075</c:v>
+                  <c:v>272848.949</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>45273.67975</c:v>
+                  <c:v>48704.53825</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>141129.76275</c:v>
@@ -4080,19 +4080,22 @@
         <v>201</v>
       </c>
       <c r="E28">
-        <v>50</v>
+        <v>53.8</v>
+      </c>
+      <c r="F28" s="3">
+        <v>46230</v>
       </c>
       <c r="G28">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="I28">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="J28">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="K28" t="s">
         <v>205</v>
@@ -4112,22 +4115,22 @@
         <v>201</v>
       </c>
       <c r="E29">
-        <v>53.8</v>
+        <v>66.2</v>
       </c>
       <c r="F29" s="3">
-        <v>46230</v>
+        <v>46248</v>
       </c>
       <c r="G29">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="H29">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="I29">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="J29">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="K29" t="s">
         <v>205</v>
@@ -4135,7 +4138,7 @@
     </row>
     <row r="30" spans="1:11">
       <c r="A30" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B30" t="s">
         <v>55</v>
@@ -4147,22 +4150,22 @@
         <v>201</v>
       </c>
       <c r="E30">
-        <v>66.2</v>
+        <v>54.4</v>
       </c>
       <c r="F30" s="3">
-        <v>46248</v>
+        <v>46250</v>
       </c>
       <c r="G30">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H30">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="I30">
         <v>68</v>
       </c>
       <c r="J30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K30" t="s">
         <v>205</v>
@@ -4170,7 +4173,7 @@
     </row>
     <row r="31" spans="1:11">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B31" t="s">
         <v>56</v>
@@ -4182,22 +4185,22 @@
         <v>201</v>
       </c>
       <c r="E31">
-        <v>54.4</v>
+        <v>48.9</v>
       </c>
       <c r="F31" s="3">
-        <v>46250</v>
+        <v>46247</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H31">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="I31">
-        <v>68</v>
+        <v>47</v>
       </c>
       <c r="J31">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K31" t="s">
         <v>205</v>
@@ -4205,7 +4208,7 @@
     </row>
     <row r="32" spans="1:11">
       <c r="A32" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="B32" t="s">
         <v>57</v>
@@ -4217,22 +4220,22 @@
         <v>201</v>
       </c>
       <c r="E32">
-        <v>48.9</v>
+        <v>69.7</v>
       </c>
       <c r="F32" s="3">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="G32">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H32">
         <v>23</v>
       </c>
       <c r="I32">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="J32">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K32" t="s">
         <v>205</v>
@@ -4240,7 +4243,7 @@
     </row>
     <row r="33" spans="1:11">
       <c r="A33" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B33" t="s">
         <v>58</v>
@@ -4252,7 +4255,7 @@
         <v>201</v>
       </c>
       <c r="E33">
-        <v>69.7</v>
+        <v>47.2</v>
       </c>
       <c r="F33" s="3">
         <v>46248</v>
@@ -4261,10 +4264,10 @@
         <v>2</v>
       </c>
       <c r="H33">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I33">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="J33">
         <v>1</v>
@@ -4287,7 +4290,7 @@
         <v>201</v>
       </c>
       <c r="E34">
-        <v>47.2</v>
+        <v>49.1</v>
       </c>
       <c r="F34" s="3">
         <v>46248</v>
@@ -4296,7 +4299,7 @@
         <v>2</v>
       </c>
       <c r="H34">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I34">
         <v>53</v>
@@ -4325,10 +4328,10 @@
         <v>49.1</v>
       </c>
       <c r="F35" s="3">
-        <v>46248</v>
+        <v>46245</v>
       </c>
       <c r="G35">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H35">
         <v>26</v>
@@ -4337,7 +4340,7 @@
         <v>53</v>
       </c>
       <c r="J35">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K35" t="s">
         <v>205</v>
@@ -4357,22 +4360,22 @@
         <v>201</v>
       </c>
       <c r="E36">
-        <v>49.1</v>
+        <v>50</v>
       </c>
       <c r="F36" s="3">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H36">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="I36">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="J36">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K36" t="s">
         <v>205</v>
@@ -4395,10 +4398,10 @@
         <v>50</v>
       </c>
       <c r="F37" s="3">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="G37">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37">
         <v>2</v>
@@ -4407,7 +4410,7 @@
         <v>4</v>
       </c>
       <c r="J37">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K37" t="s">
         <v>205</v>
@@ -4430,10 +4433,10 @@
         <v>50</v>
       </c>
       <c r="F38" s="3">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="G38">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H38">
         <v>2</v>
@@ -4442,7 +4445,7 @@
         <v>4</v>
       </c>
       <c r="J38">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K38" t="s">
         <v>205</v>
@@ -4462,7 +4465,7 @@
         <v>201</v>
       </c>
       <c r="E39">
-        <v>50</v>
+        <v>50.9</v>
       </c>
       <c r="F39" s="3">
         <v>46247</v>
@@ -4471,10 +4474,10 @@
         <v>3</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="I39">
-        <v>4</v>
+        <v>53</v>
       </c>
       <c r="J39">
         <v>2</v>
@@ -4497,22 +4500,22 @@
         <v>201</v>
       </c>
       <c r="E40">
-        <v>50.9</v>
+        <v>52.9</v>
       </c>
       <c r="F40" s="3">
-        <v>46247</v>
+        <v>46245</v>
       </c>
       <c r="G40">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H40">
         <v>27</v>
       </c>
       <c r="I40">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="J40">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K40" t="s">
         <v>205</v>
@@ -4532,22 +4535,22 @@
         <v>201</v>
       </c>
       <c r="E41">
-        <v>52.9</v>
+        <v>60.4</v>
       </c>
       <c r="F41" s="3">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="G41">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H41">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="I41">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="J41">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K41" t="s">
         <v>205</v>
@@ -4567,22 +4570,22 @@
         <v>201</v>
       </c>
       <c r="E42">
-        <v>60.4</v>
+        <v>61.5</v>
       </c>
       <c r="F42" s="3">
-        <v>46247</v>
+        <v>46246</v>
       </c>
       <c r="G42">
+        <v>4</v>
+      </c>
+      <c r="H42">
+        <v>24</v>
+      </c>
+      <c r="I42">
+        <v>39</v>
+      </c>
+      <c r="J42">
         <v>3</v>
-      </c>
-      <c r="H42">
-        <v>32</v>
-      </c>
-      <c r="I42">
-        <v>53</v>
-      </c>
-      <c r="J42">
-        <v>2</v>
       </c>
       <c r="K42" t="s">
         <v>205</v>
@@ -4602,22 +4605,22 @@
         <v>201</v>
       </c>
       <c r="E43">
-        <v>61.5</v>
+        <v>62.3</v>
       </c>
       <c r="F43" s="3">
-        <v>46246</v>
+        <v>46241</v>
       </c>
       <c r="G43">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H43">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="I43">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="J43">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K43" t="s">
         <v>205</v>
@@ -4625,7 +4628,7 @@
     </row>
     <row r="44" spans="1:11">
       <c r="A44" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B44" t="s">
         <v>69</v>
@@ -4637,22 +4640,22 @@
         <v>201</v>
       </c>
       <c r="E44">
-        <v>62.3</v>
+        <v>50</v>
       </c>
       <c r="F44" s="3">
-        <v>46241</v>
+        <v>46247</v>
       </c>
       <c r="G44">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H44">
-        <v>33</v>
+        <v>13</v>
       </c>
       <c r="I44">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="J44">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K44" t="s">
         <v>205</v>
@@ -4672,22 +4675,22 @@
         <v>201</v>
       </c>
       <c r="E45">
-        <v>50</v>
+        <v>57.7</v>
       </c>
       <c r="F45" s="3">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="G45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H45">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I45">
         <v>26</v>
       </c>
       <c r="J45">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K45" t="s">
         <v>205</v>
@@ -4695,7 +4698,7 @@
     </row>
     <row r="46" spans="1:11">
       <c r="A46" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B46" t="s">
         <v>71</v>
@@ -4707,22 +4710,22 @@
         <v>201</v>
       </c>
       <c r="E46">
-        <v>57.7</v>
+        <v>50</v>
       </c>
       <c r="F46" s="3">
-        <v>46248</v>
+        <v>46247</v>
       </c>
       <c r="G46">
+        <v>3</v>
+      </c>
+      <c r="H46">
+        <v>3</v>
+      </c>
+      <c r="I46">
+        <v>6</v>
+      </c>
+      <c r="J46">
         <v>2</v>
-      </c>
-      <c r="H46">
-        <v>15</v>
-      </c>
-      <c r="I46">
-        <v>26</v>
-      </c>
-      <c r="J46">
-        <v>1</v>
       </c>
       <c r="K46" t="s">
         <v>205</v>
@@ -4777,7 +4780,7 @@
         <v>201</v>
       </c>
       <c r="E48">
-        <v>50</v>
+        <v>66.7</v>
       </c>
       <c r="F48" s="3">
         <v>46247</v>
@@ -4786,7 +4789,7 @@
         <v>3</v>
       </c>
       <c r="H48">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I48">
         <v>6</v>
@@ -4800,7 +4803,7 @@
     </row>
     <row r="49" spans="1:11">
       <c r="A49" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="B49" t="s">
         <v>74</v>
@@ -4809,33 +4812,33 @@
         <v>159</v>
       </c>
       <c r="D49" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E49">
-        <v>66.7</v>
+        <v>20.5</v>
       </c>
       <c r="F49" s="3">
-        <v>46247</v>
+        <v>46219</v>
       </c>
       <c r="G49">
-        <v>3</v>
+        <v>31</v>
       </c>
       <c r="H49">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="I49">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="J49">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="K49" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="50" spans="1:11">
       <c r="A50" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B50" t="s">
         <v>75</v>
@@ -4847,22 +4850,22 @@
         <v>202</v>
       </c>
       <c r="E50">
-        <v>20.5</v>
+        <v>23.5</v>
       </c>
       <c r="F50" s="3">
-        <v>46219</v>
+        <v>46245</v>
       </c>
       <c r="G50">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="H50">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="I50">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="J50">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="K50" t="s">
         <v>206</v>
@@ -4882,22 +4885,22 @@
         <v>202</v>
       </c>
       <c r="E51">
-        <v>23.5</v>
+        <v>27.9</v>
       </c>
       <c r="F51" s="3">
-        <v>46245</v>
+        <v>46247</v>
       </c>
       <c r="G51">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H51">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I51">
         <v>68</v>
       </c>
       <c r="J51">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K51" t="s">
         <v>206</v>
@@ -4917,7 +4920,7 @@
         <v>202</v>
       </c>
       <c r="E52">
-        <v>27.9</v>
+        <v>29.4</v>
       </c>
       <c r="F52" s="3">
         <v>46247</v>
@@ -4926,7 +4929,7 @@
         <v>3</v>
       </c>
       <c r="H52">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I52">
         <v>68</v>
@@ -4952,22 +4955,22 @@
         <v>202</v>
       </c>
       <c r="E53">
-        <v>29.4</v>
+        <v>33.8</v>
       </c>
       <c r="F53" s="3">
-        <v>46247</v>
+        <v>46248</v>
       </c>
       <c r="G53">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H53">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="I53">
         <v>68</v>
       </c>
       <c r="J53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K53" t="s">
         <v>206</v>
@@ -4975,7 +4978,7 @@
     </row>
     <row r="54" spans="1:11">
       <c r="A54" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B54" t="s">
         <v>79</v>
@@ -4987,22 +4990,22 @@
         <v>202</v>
       </c>
       <c r="E54">
-        <v>33.8</v>
+        <v>41.2</v>
       </c>
       <c r="F54" s="3">
-        <v>46248</v>
+        <v>46250</v>
       </c>
       <c r="G54">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H54">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I54">
         <v>68</v>
       </c>
       <c r="J54">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K54" t="s">
         <v>206</v>
@@ -5010,7 +5013,7 @@
     </row>
     <row r="55" spans="1:11">
       <c r="A55" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B55" t="s">
         <v>80</v>
@@ -5022,22 +5025,22 @@
         <v>202</v>
       </c>
       <c r="E55">
-        <v>41.2</v>
+        <v>10.3</v>
       </c>
       <c r="F55" s="3">
-        <v>46250</v>
+        <v>46231</v>
       </c>
       <c r="G55">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="H55">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="I55">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="J55">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K55" t="s">
         <v>206</v>
@@ -5057,22 +5060,22 @@
         <v>202</v>
       </c>
       <c r="E56">
-        <v>10.3</v>
+        <v>17</v>
       </c>
       <c r="F56" s="3">
-        <v>46231</v>
+        <v>46245</v>
       </c>
       <c r="G56">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="H56">
+        <v>9</v>
+      </c>
+      <c r="I56">
+        <v>53</v>
+      </c>
+      <c r="J56">
         <v>4</v>
-      </c>
-      <c r="I56">
-        <v>39</v>
-      </c>
-      <c r="J56">
-        <v>14</v>
       </c>
       <c r="K56" t="s">
         <v>206</v>
@@ -5092,22 +5095,22 @@
         <v>202</v>
       </c>
       <c r="E57">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F57" s="3">
-        <v>46245</v>
+        <v>46246</v>
       </c>
       <c r="G57">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H57">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="I57">
-        <v>53</v>
+        <v>4</v>
       </c>
       <c r="J57">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K57" t="s">
         <v>206</v>
@@ -5165,10 +5168,10 @@
         <v>25</v>
       </c>
       <c r="F59" s="3">
-        <v>46246</v>
+        <v>46248</v>
       </c>
       <c r="G59">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H59">
         <v>1</v>
@@ -5177,7 +5180,7 @@
         <v>4</v>
       </c>
       <c r="J59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K59" t="s">
         <v>206</v>
@@ -5197,22 +5200,22 @@
         <v>202</v>
       </c>
       <c r="E60">
-        <v>25</v>
+        <v>28.2</v>
       </c>
       <c r="F60" s="3">
-        <v>46248</v>
+        <v>46237</v>
       </c>
       <c r="G60">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="H60">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="I60">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="J60">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="K60" t="s">
         <v>206</v>
@@ -5232,22 +5235,22 @@
         <v>202</v>
       </c>
       <c r="E61">
-        <v>28.2</v>
+        <v>41.5</v>
       </c>
       <c r="F61" s="3">
-        <v>46237</v>
+        <v>46249</v>
       </c>
       <c r="G61">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="H61">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I61">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="J61">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K61" t="s">
         <v>206</v>
@@ -5267,22 +5270,22 @@
         <v>202</v>
       </c>
       <c r="E62">
-        <v>41.5</v>
+        <v>43.4</v>
       </c>
       <c r="F62" s="3">
-        <v>46249</v>
+        <v>46223</v>
       </c>
       <c r="G62">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="H62">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I62">
         <v>53</v>
       </c>
       <c r="J62">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K62" t="s">
         <v>206</v>
@@ -5302,22 +5305,22 @@
         <v>202</v>
       </c>
       <c r="E63">
-        <v>43.4</v>
+        <v>43.6</v>
       </c>
       <c r="F63" s="3">
-        <v>46223</v>
+        <v>46248</v>
       </c>
       <c r="G63">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="H63">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="I63">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="J63">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="K63" t="s">
         <v>206</v>
@@ -5325,7 +5328,7 @@
     </row>
     <row r="64" spans="1:11">
       <c r="A64" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B64" t="s">
         <v>89</v>
@@ -5337,22 +5340,22 @@
         <v>202</v>
       </c>
       <c r="E64">
-        <v>43.6</v>
+        <v>14.3</v>
       </c>
       <c r="F64" s="3">
-        <v>46248</v>
+        <v>46244</v>
       </c>
       <c r="G64">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H64">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="I64">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="J64">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K64" t="s">
         <v>206</v>
@@ -5360,7 +5363,7 @@
     </row>
     <row r="65" spans="1:11">
       <c r="A65" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B65" t="s">
         <v>90</v>
@@ -5372,22 +5375,22 @@
         <v>202</v>
       </c>
       <c r="E65">
-        <v>14.3</v>
+        <v>11.5</v>
       </c>
       <c r="F65" s="3">
-        <v>46244</v>
+        <v>46246</v>
       </c>
       <c r="G65">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H65">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I65">
-        <v>7</v>
+        <v>26</v>
       </c>
       <c r="J65">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K65" t="s">
         <v>206</v>
@@ -5410,10 +5413,10 @@
         <v>11.5</v>
       </c>
       <c r="F66" s="3">
-        <v>46246</v>
+        <v>46240</v>
       </c>
       <c r="G66">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H66">
         <v>3</v>
@@ -5422,7 +5425,7 @@
         <v>26</v>
       </c>
       <c r="J66">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="K66" t="s">
         <v>206</v>
@@ -5445,10 +5448,10 @@
         <v>11.5</v>
       </c>
       <c r="F67" s="3">
-        <v>46240</v>
+        <v>46241</v>
       </c>
       <c r="G67">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H67">
         <v>3</v>
@@ -5457,7 +5460,7 @@
         <v>26</v>
       </c>
       <c r="J67">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K67" t="s">
         <v>206</v>
@@ -5477,22 +5480,22 @@
         <v>202</v>
       </c>
       <c r="E68">
-        <v>11.5</v>
+        <v>19.2</v>
       </c>
       <c r="F68" s="3">
-        <v>46241</v>
+        <v>46245</v>
       </c>
       <c r="G68">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H68">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I68">
         <v>26</v>
       </c>
       <c r="J68">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K68" t="s">
         <v>206</v>
@@ -5515,10 +5518,10 @@
         <v>19.2</v>
       </c>
       <c r="F69" s="3">
-        <v>46245</v>
+        <v>46238</v>
       </c>
       <c r="G69">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="H69">
         <v>5</v>
@@ -5527,7 +5530,7 @@
         <v>26</v>
       </c>
       <c r="J69">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="K69" t="s">
         <v>206</v>
@@ -5547,22 +5550,22 @@
         <v>202</v>
       </c>
       <c r="E70">
-        <v>19.2</v>
+        <v>34.6</v>
       </c>
       <c r="F70" s="3">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="G70">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="H70">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="I70">
         <v>26</v>
       </c>
       <c r="J70">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="K70" t="s">
         <v>206</v>
@@ -5570,7 +5573,7 @@
     </row>
     <row r="71" spans="1:11">
       <c r="A71" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B71" t="s">
         <v>96</v>
@@ -5579,28 +5582,25 @@
         <v>181</v>
       </c>
       <c r="D71" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E71">
-        <v>34.6</v>
-      </c>
-      <c r="F71" s="3">
-        <v>46245</v>
+        <v>0</v>
       </c>
       <c r="G71">
-        <v>5</v>
+        <v>17</v>
       </c>
       <c r="H71">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="I71">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="J71">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="K71" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -5617,19 +5617,22 @@
         <v>203</v>
       </c>
       <c r="E72">
-        <v>0</v>
+        <v>2.6</v>
+      </c>
+      <c r="F72" s="3">
+        <v>46249</v>
       </c>
       <c r="G72">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="H72">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I72">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="J72">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K72" t="s">
         <v>207</v>
@@ -5637,7 +5640,7 @@
     </row>
     <row r="73" spans="1:11">
       <c r="A73" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B73" t="s">
         <v>98</v>
@@ -5649,22 +5652,19 @@
         <v>203</v>
       </c>
       <c r="E73">
-        <v>2.6</v>
-      </c>
-      <c r="F73" s="3">
-        <v>46249</v>
+        <v>0</v>
       </c>
       <c r="G73">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="H73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I73">
-        <v>39</v>
+        <v>68</v>
       </c>
       <c r="J73">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="K73" t="s">
         <v>207</v>
@@ -5672,7 +5672,7 @@
     </row>
     <row r="74" spans="1:11">
       <c r="A74" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B74" t="s">
         <v>99</v>
@@ -5684,19 +5684,22 @@
         <v>203</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>3.8</v>
+      </c>
+      <c r="F74" s="3">
+        <v>46247</v>
       </c>
       <c r="G74">
-        <v>95</v>
+        <v>3</v>
       </c>
       <c r="H74">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I74">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="J74">
-        <v>68</v>
+        <v>2</v>
       </c>
       <c r="K74" t="s">
         <v>207</v>
@@ -5704,7 +5707,7 @@
     </row>
     <row r="75" spans="1:11">
       <c r="A75" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B75" t="s">
         <v>100</v>
@@ -5713,28 +5716,25 @@
         <v>185</v>
       </c>
       <c r="D75" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E75">
-        <v>3.8</v>
-      </c>
-      <c r="F75" s="3">
-        <v>46247</v>
+        <v>0</v>
       </c>
       <c r="G75">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H75">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I75">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="J75">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K75" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -6211,10 +6211,10 @@
         <v>201</v>
       </c>
       <c r="B6">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6">
-        <v>54.6</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -6244,7 +6244,7 @@
         <v>204</v>
       </c>
       <c r="B9">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -6384,30 +6384,30 @@
     </row>
     <row r="11" spans="1:4">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B11">
         <v>7</v>
       </c>
       <c r="C11">
-        <v>40.8</v>
+        <v>37.6</v>
       </c>
       <c r="D11">
-        <v>16.1</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12">
         <v>7</v>
       </c>
       <c r="C12">
-        <v>37.6</v>
+        <v>33.6</v>
       </c>
       <c r="D12">
-        <v>25.6</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -6546,16 +6546,16 @@
         <v>220</v>
       </c>
       <c r="C8">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" s="4">
-        <v>5040</v>
+        <v>4800</v>
       </c>
       <c r="E8" s="4">
-        <v>104004.2029166667</v>
+        <v>100573.3444166667</v>
       </c>
       <c r="F8">
-        <v>22.5</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -6606,16 +6606,16 @@
         <v>222</v>
       </c>
       <c r="C11">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D11" s="4">
-        <v>3120</v>
+        <v>3360</v>
       </c>
       <c r="E11" s="4">
-        <v>45273.67975</v>
+        <v>48704.53825</v>
       </c>
       <c r="F11">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -6663,16 +6663,16 @@
         <v>220</v>
       </c>
       <c r="B15">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C15">
-        <v>276279.8075</v>
+        <v>272848.949</v>
       </c>
       <c r="D15" s="4">
-        <v>14640</v>
+        <v>14400</v>
       </c>
       <c r="E15" s="4">
-        <v>59.7</v>
+        <v>59</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -6680,16 +6680,16 @@
         <v>222</v>
       </c>
       <c r="B16">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16">
-        <v>45273.67975</v>
+        <v>48704.53825</v>
       </c>
       <c r="D16" s="4">
-        <v>3120</v>
+        <v>3360</v>
       </c>
       <c r="E16" s="4">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -7398,10 +7398,10 @@
     </row>
     <row r="5" spans="1:40">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C5" t="s">
         <v>262</v>
@@ -7517,10 +7517,10 @@
     </row>
     <row r="6" spans="1:40">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C6" t="s">
         <v>262</v>
@@ -7636,10 +7636,10 @@
     </row>
     <row r="7" spans="1:40">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B7" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C7" t="s">
         <v>262</v>
@@ -7755,10 +7755,10 @@
     </row>
     <row r="8" spans="1:40">
       <c r="A8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C8" t="s">
         <v>262</v>
@@ -7874,10 +7874,10 @@
     </row>
     <row r="9" spans="1:40">
       <c r="A9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C9" t="s">
         <v>262</v>
@@ -8112,10 +8112,10 @@
     </row>
     <row r="11" spans="1:40">
       <c r="A11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C11" t="s">
         <v>262</v>
@@ -8151,10 +8151,10 @@
         <v>46155</v>
       </c>
       <c r="N11" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="O11" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q11">
         <v>0</v>
@@ -8466,10 +8466,10 @@
     </row>
     <row r="14" spans="1:40">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C14" t="s">
         <v>262</v>
@@ -8585,10 +8585,10 @@
     </row>
     <row r="15" spans="1:40">
       <c r="A15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C15" t="s">
         <v>262</v>
@@ -8704,10 +8704,10 @@
     </row>
     <row r="16" spans="1:40">
       <c r="A16" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C16" t="s">
         <v>263</v>
@@ -9061,10 +9061,10 @@
     </row>
     <row r="19" spans="1:40">
       <c r="A19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C19" t="s">
         <v>263</v>
@@ -9418,10 +9418,10 @@
     </row>
     <row r="22" spans="1:40">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B22" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C22" t="s">
         <v>263</v>
@@ -9537,10 +9537,10 @@
     </row>
     <row r="23" spans="1:40">
       <c r="A23" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C23" t="s">
         <v>263</v>
@@ -9775,10 +9775,10 @@
     </row>
     <row r="25" spans="1:40">
       <c r="A25" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B25" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C25" t="s">
         <v>264</v>
@@ -10132,10 +10132,10 @@
     </row>
     <row r="28" spans="1:40">
       <c r="A28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B28" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C28" t="s">
         <v>264</v>
@@ -10251,10 +10251,10 @@
     </row>
     <row r="29" spans="1:40">
       <c r="A29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B29" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C29" t="s">
         <v>264</v>
@@ -10370,10 +10370,10 @@
     </row>
     <row r="30" spans="1:40">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B30" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C30" t="s">
         <v>264</v>
@@ -10489,10 +10489,10 @@
     </row>
     <row r="31" spans="1:40">
       <c r="A31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B31" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C31" t="s">
         <v>264</v>
@@ -10608,10 +10608,10 @@
     </row>
     <row r="32" spans="1:40">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C32" t="s">
         <v>265</v>
@@ -10846,10 +10846,10 @@
     </row>
     <row r="34" spans="1:40">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B34" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C34" t="s">
         <v>267</v>
@@ -10965,10 +10965,10 @@
     </row>
     <row r="35" spans="1:40">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B35" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C35" t="s">
         <v>268</v>
@@ -11560,10 +11560,10 @@
     </row>
     <row r="40" spans="1:40">
       <c r="A40" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B40" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C40" t="s">
         <v>268</v>
@@ -11679,10 +11679,10 @@
     </row>
     <row r="41" spans="1:40">
       <c r="A41" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B41" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C41" t="s">
         <v>268</v>
@@ -11798,10 +11798,10 @@
     </row>
     <row r="42" spans="1:40">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B42" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C42" t="s">
         <v>268</v>
@@ -12036,10 +12036,10 @@
     </row>
     <row r="44" spans="1:40">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B44" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C44" t="s">
         <v>268</v>
@@ -12155,10 +12155,10 @@
     </row>
     <row r="45" spans="1:40">
       <c r="A45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C45" t="s">
         <v>268</v>
@@ -12274,10 +12274,10 @@
     </row>
     <row r="46" spans="1:40">
       <c r="A46" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B46" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C46" t="s">
         <v>268</v>
@@ -12631,10 +12631,10 @@
     </row>
     <row r="49" spans="1:40">
       <c r="A49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B49" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C49" t="s">
         <v>269</v>
@@ -12869,10 +12869,10 @@
     </row>
     <row r="51" spans="1:40">
       <c r="A51" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B51" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C51" t="s">
         <v>267</v>
@@ -12988,10 +12988,10 @@
     </row>
     <row r="52" spans="1:40">
       <c r="A52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B52" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C52" t="s">
         <v>267</v>
@@ -13107,10 +13107,10 @@
     </row>
     <row r="53" spans="1:40">
       <c r="A53" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B53" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C53" t="s">
         <v>267</v>
@@ -13226,10 +13226,10 @@
     </row>
     <row r="54" spans="1:40">
       <c r="A54" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B54" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C54" t="s">
         <v>267</v>
@@ -13345,10 +13345,10 @@
     </row>
     <row r="55" spans="1:40">
       <c r="A55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C55" t="s">
         <v>270</v>
@@ -13464,10 +13464,10 @@
     </row>
     <row r="56" spans="1:40">
       <c r="A56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B56" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C56" t="s">
         <v>270</v>
@@ -13583,10 +13583,10 @@
     </row>
     <row r="57" spans="1:40">
       <c r="A57" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B57" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C57" t="s">
         <v>270</v>
@@ -13702,10 +13702,10 @@
     </row>
     <row r="58" spans="1:40">
       <c r="A58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B58" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C58" t="s">
         <v>270</v>
@@ -13821,10 +13821,10 @@
     </row>
     <row r="59" spans="1:40">
       <c r="A59" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B59" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C59" t="s">
         <v>270</v>
@@ -14062,10 +14062,10 @@
     </row>
     <row r="61" spans="1:40">
       <c r="A61" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B61" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C61" t="s">
         <v>271</v>
@@ -14101,10 +14101,10 @@
         <v>46233</v>
       </c>
       <c r="N61" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O61" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q61">
         <v>0</v>
@@ -14178,10 +14178,10 @@
     </row>
     <row r="62" spans="1:40">
       <c r="A62" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B62" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C62" t="s">
         <v>272</v>
@@ -14416,10 +14416,10 @@
     </row>
     <row r="64" spans="1:40">
       <c r="A64" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B64" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C64" t="s">
         <v>273</v>
@@ -14651,10 +14651,10 @@
     </row>
     <row r="66" spans="1:40">
       <c r="A66" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B66" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C66" t="s">
         <v>273</v>
@@ -14770,10 +14770,10 @@
     </row>
     <row r="67" spans="1:40">
       <c r="A67" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B67" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C67" t="s">
         <v>273</v>
@@ -14928,10 +14928,10 @@
         <v>46245</v>
       </c>
       <c r="N68" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O68" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q68">
         <v>0</v>
@@ -15124,10 +15124,10 @@
     </row>
     <row r="70" spans="1:40">
       <c r="A70" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B70" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C70" t="s">
         <v>274</v>
@@ -15243,10 +15243,10 @@
     </row>
     <row r="71" spans="1:40">
       <c r="A71" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B71" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C71" t="s">
         <v>274</v>
@@ -15362,10 +15362,10 @@
     </row>
     <row r="72" spans="1:40">
       <c r="A72" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B72" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C72" t="s">
         <v>274</v>
@@ -15481,10 +15481,10 @@
     </row>
     <row r="73" spans="1:40">
       <c r="A73" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B73" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C73" t="s">
         <v>274</v>
@@ -15639,10 +15639,10 @@
         <v>46245</v>
       </c>
       <c r="N74" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O74" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q74">
         <v>0</v>
@@ -15832,10 +15832,10 @@
     </row>
     <row r="76" spans="1:40">
       <c r="A76" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B76" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C76" t="s">
         <v>274</v>
@@ -15990,10 +15990,10 @@
         <v>46245</v>
       </c>
       <c r="N77" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O77" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q77">
         <v>0</v>
@@ -16106,10 +16106,10 @@
         <v>46245</v>
       </c>
       <c r="N78" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O78" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q78">
         <v>0</v>
@@ -16454,10 +16454,10 @@
         <v>46245</v>
       </c>
       <c r="N81" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O81" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q81">
         <v>0</v>
@@ -16531,10 +16531,10 @@
     </row>
     <row r="82" spans="1:40">
       <c r="A82" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B82" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C82" t="s">
         <v>274</v>
@@ -16689,10 +16689,10 @@
         <v>46245</v>
       </c>
       <c r="N83" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O83" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q83">
         <v>0</v>
@@ -17040,10 +17040,10 @@
         <v>46245</v>
       </c>
       <c r="N86" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O86" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q86">
         <v>0</v>
@@ -17117,10 +17117,10 @@
     </row>
     <row r="87" spans="1:40">
       <c r="A87" t="s">
-        <v>53</v>
+        <v>100</v>
       </c>
       <c r="B87" t="s">
-        <v>138</v>
+        <v>185</v>
       </c>
       <c r="C87" t="s">
         <v>274</v>
@@ -17156,19 +17156,19 @@
         <v>46245</v>
       </c>
       <c r="N87" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O87" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q87">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R87">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S87">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T87">
         <v>0</v>
@@ -17210,16 +17210,16 @@
         <v>5</v>
       </c>
       <c r="AG87">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="AH87" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="AI87">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ87" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="AL87">
         <v>85</v>
@@ -17394,10 +17394,10 @@
         <v>46251</v>
       </c>
       <c r="N89" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="O89" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="Q89">
         <v>0</v>

</xml_diff>